<commit_message>
Clean stale JD generations; archive history; fix JD-aware highlighting
- Move old JD generations (20260917, 20260919) and their sources into archive/
- Archive stale outputs (tailored, preview, 6 Interview Prep, cover_letters, interview_prep)
- Keep only active JD 20260920-0013 in custom_cv / job_descriptions / Job Applications
- Remove empty Temp/, stray .pyc, temp scratch (tmp_compile.sh, tmp_variant_import.typ), debug module
- Fix engine.py _jd_aware_highlight: correct seen/add ordering, add missing important flags
- Preserve hidden .generation_debug.log for later process improvement
</commit_message>
<xml_diff>
--- a/application_monitoring/Application_Tracker.xlsx
+++ b/application_monitoring/Application_Tracker.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -924,6 +924,152 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CV-20260918-0011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Financial Modelling</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Job Description (text)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(pasted text)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>job_descriptions\CV-20260918-0011.txt</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>C:\MyDev\MyCV\Job Applications\20260918 - Unknown_Company - Unknown_Position\CV-20260918-0011_RM1.docx</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Generated 20260918: 0 CV PDF(s) + 0 cover letter(s) + 0 interview prep(s) + 1 recruiter message(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CV-20260919-0012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Manages Large</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Lead BI &amp; Analytics Consultant</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>job_descriptions\CV-20260919-0012.txt</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>C:\MyDev\MyCV\custom_cv\CV-20260919-0012_CV0012.pdf; C:\MyDev\MyCV\Job Applications\20260919 - Unknown_Company - Unknown_Position\CV-20260919-0012_RM1.docx</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Generated 20260920: 1 CV PDF(s) + 0 cover letter(s) + 0 interview prep(s) + 1 recruiter message(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CV-20260920-0013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Align With Business Objectives</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Job Description (text)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(pasted text)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>job_descriptions\CV-20260920-0013.txt</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>C:\MyDev\MyCV\20260920 - Align With Business Objectives - Chief Growth &amp; Transformation Officer\CV-20260920-0013_CV1.pdf; C:\MyDev\MyCV\custom_cv\CV-20260920-0013_CV0013.pdf; C:\MyDev\MyCV\Job Applications\20260920 - Align_With_Business_Objectives - Unknown_Position\CV-20260920-0013_RM1.docx</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Generated 20260920: 2 CV PDF(s) + 0 cover letter(s) + 0 interview prep(s) + 1 recruiter message(s)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>